<commit_message>
25/05/2026 h0900: 4 posters loaded on INDICO
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nontr\Documents\pisa-conf\ftdm26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1CCB70C-E750-4E22-B4F5-FF466556DB79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B86A5DEE-A63A-44C5-8B05-93C9AC7F0331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="81">
   <si>
     <t>Key</t>
   </si>
@@ -46,10 +46,7 @@
     <t>Forum on Tracking Detector Mechanics 2026</t>
   </si>
   <si>
-    <t>2026-06-01</t>
-  </si>
-  <si>
-    <t>2026-06-05</t>
+    <t>Hotel Hermitage</t>
   </si>
   <si>
     <t>Session ID</t>
@@ -67,12 +64,6 @@
     <t>Forum Poster Session</t>
   </si>
   <si>
-    <t>2026-06-02 15:00:00</t>
-  </si>
-  <si>
-    <t>2026-06-02 15:30:00</t>
-  </si>
-  <si>
     <t>Hostname</t>
   </si>
   <si>
@@ -193,10 +184,88 @@
     <t>Deutsches Elektronen-Synchrotron  (DE)</t>
   </si>
   <si>
-    <t>La Biodola</t>
+    <t>pi5pm1</t>
+  </si>
+  <si>
+    <t>pi5pm2</t>
+  </si>
+  <si>
+    <t>pi5pm3</t>
+  </si>
+  <si>
+    <t>pi5pm4</t>
+  </si>
+  <si>
+    <t>pi5pm5</t>
+  </si>
+  <si>
+    <t>pi5pm6</t>
+  </si>
+  <si>
+    <t>pi5pm7</t>
+  </si>
+  <si>
+    <t>pi5pm8</t>
+  </si>
+  <si>
+    <t>pi5pm9</t>
+  </si>
+  <si>
+    <t>pi5pm10</t>
+  </si>
+  <si>
+    <t>pi5pm11</t>
   </si>
   <si>
     <t>pi5pm12</t>
+  </si>
+  <si>
+    <t>pi5pm13</t>
+  </si>
+  <si>
+    <t>pi5pm14</t>
+  </si>
+  <si>
+    <t>pi5pm15</t>
+  </si>
+  <si>
+    <t>pi5pm16</t>
+  </si>
+  <si>
+    <t>pi5pm17</t>
+  </si>
+  <si>
+    <t>pi5pm18</t>
+  </si>
+  <si>
+    <t>pi5pm19</t>
+  </si>
+  <si>
+    <t>pi5pm20</t>
+  </si>
+  <si>
+    <t>pi5pm21</t>
+  </si>
+  <si>
+    <t>pi5pm22</t>
+  </si>
+  <si>
+    <t>pi5pm23</t>
+  </si>
+  <si>
+    <t>pi5pm24</t>
+  </si>
+  <si>
+    <t>pi5pm25</t>
+  </si>
+  <si>
+    <t>pi5pm26</t>
+  </si>
+  <si>
+    <t>pi5pm27</t>
+  </si>
+  <si>
+    <t>pi5pm28</t>
   </si>
 </sst>
 </file>
@@ -255,11 +324,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -592,23 +663,23 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>56</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
-        <v>7</v>
+      <c r="B4" s="2">
+        <v>46174</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" t="s">
-        <v>8</v>
+      <c r="B5" s="2">
+        <v>46178</v>
       </c>
     </row>
   </sheetData>
@@ -628,16 +699,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
@@ -645,13 +716,13 @@
         <v>665057</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D2" t="s">
-        <v>15</v>
+        <v>12</v>
+      </c>
+      <c r="C2" s="3">
+        <v>46174.291666666664</v>
+      </c>
+      <c r="D2" s="3">
+        <v>46178.833333333336</v>
       </c>
     </row>
   </sheetData>
@@ -661,7 +732,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20.73046875" customWidth="1"/>
@@ -669,18 +740,234 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
         <v>57</v>
       </c>
-      <c r="B2">
+      <c r="B6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>64</v>
+      </c>
+      <c r="B13">
         <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>66</v>
+      </c>
+      <c r="B15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>69</v>
+      </c>
+      <c r="B18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>70</v>
+      </c>
+      <c r="B19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>73</v>
+      </c>
+      <c r="B22">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>74</v>
+      </c>
+      <c r="B23">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>75</v>
+      </c>
+      <c r="B24">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>76</v>
+      </c>
+      <c r="B25">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>77</v>
+      </c>
+      <c r="B26">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>78</v>
+      </c>
+      <c r="B27">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>80</v>
+      </c>
+      <c r="B29">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -701,202 +988,175 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>19</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>13</v>
       </c>
-      <c r="B2">
-        <v>12</v>
-      </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>36</v>
       </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>42</v>
       </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>50</v>
       </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F5" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>56</v>
       </c>
-      <c r="B6">
-        <v>4</v>
-      </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>61</v>
       </c>
-      <c r="B7">
-        <v>5</v>
-      </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>67</v>
       </c>
-      <c r="B8">
-        <v>6</v>
-      </c>
       <c r="C8" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>70</v>
       </c>
-      <c r="B9">
-        <v>7</v>
-      </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E9" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>87</v>
       </c>
-      <c r="B10">
-        <v>8</v>
-      </c>
       <c r="C10" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
25052026 h1400: 5/7 posters on INDICO
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nontr\Documents\pisa-conf\ftdm26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B86A5DEE-A63A-44C5-8B05-93C9AC7F0331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC57086A-481F-46E3-81BA-F26470B5E957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="79">
   <si>
     <t>Key</t>
   </si>
@@ -94,9 +94,6 @@
     <t>Thermal Performance and Radiation Tolerance of Adhesives for the CMS Phase-2 Pixel Barrel Mechanics</t>
   </si>
   <si>
-    <t>Vibration mitigation: cantilever spring blades for vertical seismic attenuation in GW interferometers</t>
-  </si>
-  <si>
     <t>Thermal Quality Control of TB2S Ladders for the CMS Phase-2 Tracker Upgrade</t>
   </si>
   <si>
@@ -106,9 +103,6 @@
     <t>CMS capillaries production for LHC High Luminosity upgrade</t>
   </si>
   <si>
-    <t>Conceiving an anti-vibration mechanical system on the experience of the Superattenuator for Gravitational Waves detectors: present and future performance</t>
-  </si>
-  <si>
     <t>CMS Phase 2 Tracker Service Channel: Thermal Performance and Simulation Results</t>
   </si>
   <si>
@@ -121,9 +115,6 @@
     <t>Andrei</t>
   </si>
   <si>
-    <t>Leonardo</t>
-  </si>
-  <si>
     <t>Lorenzo</t>
   </si>
   <si>
@@ -133,9 +124,6 @@
     <t>Arianna</t>
   </si>
   <si>
-    <t>Franco</t>
-  </si>
-  <si>
     <t>Bartosz</t>
   </si>
   <si>
@@ -148,9 +136,6 @@
     <t>Starodumov</t>
   </si>
   <si>
-    <t>Lucchesi</t>
-  </si>
-  <si>
     <t>Bistoni</t>
   </si>
   <si>
@@ -160,9 +145,6 @@
     <t>Eugeni</t>
   </si>
   <si>
-    <t>Frasconi</t>
-  </si>
-  <si>
     <t>Grygiel</t>
   </si>
   <si>
@@ -175,12 +157,6 @@
     <t>Rudjer Boskovic Institute (HR)</t>
   </si>
   <si>
-    <t>INFN Pisa</t>
-  </si>
-  <si>
-    <t>Universita e INFN, Perugia (IT)</t>
-  </si>
-  <si>
     <t>Deutsches Elektronen-Synchrotron  (DE)</t>
   </si>
   <si>
@@ -266,6 +242,24 @@
   </si>
   <si>
     <t>pi5pm28</t>
+  </si>
+  <si>
+    <t>Konrad</t>
+  </si>
+  <si>
+    <t>Wladyslaw Szczyrbak</t>
+  </si>
+  <si>
+    <t>Tadeusz Kosciuszko Cracow University of Technology (PL)</t>
+  </si>
+  <si>
+    <t>Pier Filippo</t>
+  </si>
+  <si>
+    <t>Cianchetta</t>
+  </si>
+  <si>
+    <t>Universita' e INFN, Perugia (IT)</t>
   </si>
 </sst>
 </file>
@@ -748,7 +742,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -756,7 +750,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -764,7 +758,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -772,7 +766,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -780,7 +774,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -788,7 +782,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="B7">
         <v>6</v>
@@ -796,7 +790,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B8">
         <v>7</v>
@@ -804,7 +798,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="B9">
         <v>8</v>
@@ -812,7 +806,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="B10">
         <v>9</v>
@@ -820,7 +814,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -828,7 +822,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -836,7 +830,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="B13">
         <v>12</v>
@@ -844,7 +838,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="B14">
         <v>13</v>
@@ -852,7 +846,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B15">
         <v>14</v>
@@ -860,7 +854,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B16">
         <v>15</v>
@@ -868,7 +862,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B17">
         <v>16</v>
@@ -876,7 +870,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="B18">
         <v>17</v>
@@ -884,7 +878,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="B19">
         <v>18</v>
@@ -892,7 +886,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B20">
         <v>19</v>
@@ -900,7 +894,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="B21">
         <v>20</v>
@@ -908,7 +902,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B22">
         <v>21</v>
@@ -916,7 +910,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="B23">
         <v>22</v>
@@ -924,7 +918,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="B24">
         <v>23</v>
@@ -932,7 +926,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="B25">
         <v>24</v>
@@ -940,7 +934,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="B26">
         <v>25</v>
@@ -948,7 +942,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="B27">
         <v>26</v>
@@ -956,7 +950,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="B28">
         <v>27</v>
@@ -964,7 +958,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B29">
         <v>28</v>
@@ -977,7 +971,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="12.73046875" customWidth="1"/>
@@ -1010,156 +1004,564 @@
       <c r="A2">
         <v>13</v>
       </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
       <c r="C2" t="s">
         <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F2" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3">
-        <v>36</v>
+        <v>13</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="E3" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4">
-        <v>42</v>
+        <v>13</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5">
-        <v>50</v>
+        <v>13</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" t="s">
         <v>41</v>
-      </c>
-      <c r="F5" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6">
-        <v>56</v>
+        <v>36</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" t="s">
         <v>42</v>
-      </c>
-      <c r="F6" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7">
-        <v>61</v>
+        <v>36</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D7" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="E7" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="F7" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8">
-        <v>67</v>
+        <v>36</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
         <v>35</v>
       </c>
-      <c r="E8" t="s">
-        <v>44</v>
-      </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9">
-        <v>70</v>
+        <v>36</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E9" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F9" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10">
+        <v>42</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" t="s">
+        <v>29</v>
+      </c>
+      <c r="E10" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A11">
+        <v>42</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A12">
+        <v>42</v>
+      </c>
+      <c r="B12">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A13">
+        <v>42</v>
+      </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" t="s">
+        <v>29</v>
+      </c>
+      <c r="E13" t="s">
+        <v>36</v>
+      </c>
+      <c r="F13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A14">
+        <v>56</v>
+      </c>
+      <c r="B14">
+        <v>13</v>
+      </c>
+      <c r="C14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" t="s">
+        <v>30</v>
+      </c>
+      <c r="E14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F14" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A15">
+        <v>56</v>
+      </c>
+      <c r="B15">
+        <v>14</v>
+      </c>
+      <c r="C15" t="s">
+        <v>23</v>
+      </c>
+      <c r="D15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E15" t="s">
+        <v>37</v>
+      </c>
+      <c r="F15" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A16">
+        <v>56</v>
+      </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
+      <c r="C16" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" t="s">
+        <v>76</v>
+      </c>
+      <c r="E16" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A17">
+        <v>56</v>
+      </c>
+      <c r="B17">
+        <v>16</v>
+      </c>
+      <c r="C17" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" t="s">
+        <v>77</v>
+      </c>
+      <c r="F17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A18">
+        <v>61</v>
+      </c>
+      <c r="B18">
+        <v>17</v>
+      </c>
+      <c r="C18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" t="s">
+        <v>38</v>
+      </c>
+      <c r="F18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A19">
+        <v>61</v>
+      </c>
+      <c r="B19">
+        <v>18</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" t="s">
+        <v>38</v>
+      </c>
+      <c r="F19" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A20">
+        <v>61</v>
+      </c>
+      <c r="B20">
+        <v>19</v>
+      </c>
+      <c r="C20" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E20" t="s">
+        <v>38</v>
+      </c>
+      <c r="F20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A21">
+        <v>61</v>
+      </c>
+      <c r="B21">
+        <v>20</v>
+      </c>
+      <c r="C21" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21" t="s">
+        <v>31</v>
+      </c>
+      <c r="E21" t="s">
+        <v>38</v>
+      </c>
+      <c r="F21" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A22">
+        <v>67</v>
+      </c>
+      <c r="B22">
+        <v>21</v>
+      </c>
+      <c r="C22" t="s">
+        <v>25</v>
+      </c>
+      <c r="D22" t="s">
+        <v>32</v>
+      </c>
+      <c r="E22" t="s">
+        <v>39</v>
+      </c>
+      <c r="F22" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A23">
+        <v>67</v>
+      </c>
+      <c r="B23">
+        <v>22</v>
+      </c>
+      <c r="C23" t="s">
+        <v>25</v>
+      </c>
+      <c r="D23" t="s">
+        <v>32</v>
+      </c>
+      <c r="E23" t="s">
+        <v>39</v>
+      </c>
+      <c r="F23" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A24">
+        <v>67</v>
+      </c>
+      <c r="B24">
+        <v>23</v>
+      </c>
+      <c r="C24" t="s">
+        <v>25</v>
+      </c>
+      <c r="D24" t="s">
+        <v>73</v>
+      </c>
+      <c r="E24" t="s">
+        <v>74</v>
+      </c>
+      <c r="F24" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A25">
+        <v>67</v>
+      </c>
+      <c r="B25">
+        <v>24</v>
+      </c>
+      <c r="C25" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25" t="s">
+        <v>73</v>
+      </c>
+      <c r="E25" t="s">
+        <v>74</v>
+      </c>
+      <c r="F25" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A26">
         <v>87</v>
       </c>
-      <c r="C10" t="s">
+      <c r="B26">
+        <v>25</v>
+      </c>
+      <c r="C26" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" t="s">
+        <v>40</v>
+      </c>
+      <c r="F26" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A27">
+        <v>87</v>
+      </c>
+      <c r="B27">
+        <v>26</v>
+      </c>
+      <c r="C27" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" t="s">
+        <v>33</v>
+      </c>
+      <c r="E27" t="s">
+        <v>40</v>
+      </c>
+      <c r="F27" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A28">
+        <v>87</v>
+      </c>
+      <c r="B28">
+        <v>27</v>
+      </c>
+      <c r="C28" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" t="s">
+        <v>33</v>
+      </c>
+      <c r="E28" t="s">
+        <v>40</v>
+      </c>
+      <c r="F28" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A29">
+        <v>87</v>
+      </c>
+      <c r="B29">
         <v>28</v>
       </c>
-      <c r="D10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E10" t="s">
-        <v>46</v>
-      </c>
-      <c r="F10" t="s">
-        <v>48</v>
+      <c r="C29" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" t="s">
+        <v>33</v>
+      </c>
+      <c r="E29" t="s">
+        <v>40</v>
+      </c>
+      <c r="F29" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" copies="4" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fixed date format in program
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nontr\Documents\pisa-conf\ftdm26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marco/work/git/ftdm2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC57086A-481F-46E3-81BA-F26470B5E957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695CFFF0-2F74-7E44-BA6B-E11BCEC0C44C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="83">
   <si>
     <t>Key</t>
   </si>
@@ -260,6 +260,18 @@
   </si>
   <si>
     <t>Universita' e INFN, Perugia (IT)</t>
+  </si>
+  <si>
+    <t>2026-05-29</t>
+  </si>
+  <si>
+    <t>2026-05-29 07:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-07 20:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-07</t>
   </si>
 </sst>
 </file>
@@ -323,8 +335,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -629,14 +641,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.73046875" customWidth="1"/>
-    <col min="2" max="2" width="100.73046875" customWidth="1"/>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="100.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -644,7 +656,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -652,7 +664,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -660,21 +672,24 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2">
-        <v>46174</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="B4" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2">
-        <v>46178</v>
-      </c>
+      <c r="B5" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B15" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -684,14 +699,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D2"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.73046875" customWidth="1"/>
-    <col min="2" max="2" width="100.73046875" customWidth="1"/>
-    <col min="3" max="4" width="20.73046875" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" customWidth="1"/>
+    <col min="2" max="2" width="100.6640625" customWidth="1"/>
+    <col min="3" max="4" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -705,18 +720,18 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>665057</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="3">
-        <v>46174.291666666664</v>
-      </c>
-      <c r="D2" s="3">
-        <v>46178.833333333336</v>
+      <c r="C2" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -727,12 +742,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B29"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="20.73046875" customWidth="1"/>
+    <col min="1" max="2" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
@@ -740,7 +755,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -748,7 +763,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -756,7 +771,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>47</v>
       </c>
@@ -764,7 +779,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>48</v>
       </c>
@@ -772,7 +787,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>49</v>
       </c>
@@ -780,7 +795,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>50</v>
       </c>
@@ -788,7 +803,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>51</v>
       </c>
@@ -796,7 +811,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>52</v>
       </c>
@@ -804,7 +819,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>53</v>
       </c>
@@ -812,7 +827,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>54</v>
       </c>
@@ -820,7 +835,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>55</v>
       </c>
@@ -828,7 +843,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>56</v>
       </c>
@@ -836,7 +851,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>57</v>
       </c>
@@ -844,7 +859,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>58</v>
       </c>
@@ -852,7 +867,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>59</v>
       </c>
@@ -860,7 +875,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>60</v>
       </c>
@@ -868,7 +883,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>61</v>
       </c>
@@ -876,7 +891,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>62</v>
       </c>
@@ -884,7 +899,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>63</v>
       </c>
@@ -892,7 +907,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>64</v>
       </c>
@@ -900,7 +915,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>65</v>
       </c>
@@ -908,7 +923,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>66</v>
       </c>
@@ -916,7 +931,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>67</v>
       </c>
@@ -924,7 +939,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>68</v>
       </c>
@@ -932,7 +947,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>69</v>
       </c>
@@ -940,7 +955,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>70</v>
       </c>
@@ -948,7 +963,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>71</v>
       </c>
@@ -956,7 +971,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>72</v>
       </c>
@@ -972,15 +987,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:F29"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="12.73046875" customWidth="1"/>
-    <col min="3" max="3" width="100.73046875" customWidth="1"/>
-    <col min="4" max="5" width="20.73046875" customWidth="1"/>
-    <col min="6" max="6" width="60.73046875" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.6640625" customWidth="1"/>
+    <col min="6" max="6" width="60.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -1000,7 +1015,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>13</v>
       </c>
@@ -1020,7 +1035,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>13</v>
       </c>
@@ -1040,7 +1055,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>13</v>
       </c>
@@ -1060,7 +1075,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>13</v>
       </c>
@@ -1080,7 +1095,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>36</v>
       </c>
@@ -1100,7 +1115,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>36</v>
       </c>
@@ -1120,7 +1135,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>36</v>
       </c>
@@ -1140,7 +1155,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>36</v>
       </c>
@@ -1160,7 +1175,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>42</v>
       </c>
@@ -1180,7 +1195,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>42</v>
       </c>
@@ -1200,7 +1215,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>42</v>
       </c>
@@ -1220,7 +1235,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>42</v>
       </c>
@@ -1240,7 +1255,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>56</v>
       </c>
@@ -1260,7 +1275,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>56</v>
       </c>
@@ -1280,7 +1295,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>56</v>
       </c>
@@ -1300,7 +1315,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>56</v>
       </c>
@@ -1320,7 +1335,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>61</v>
       </c>
@@ -1340,7 +1355,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>61</v>
       </c>
@@ -1360,7 +1375,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>61</v>
       </c>
@@ -1380,7 +1395,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>61</v>
       </c>
@@ -1400,7 +1415,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>67</v>
       </c>
@@ -1420,7 +1435,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>67</v>
       </c>
@@ -1440,7 +1455,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>67</v>
       </c>
@@ -1460,7 +1475,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>67</v>
       </c>
@@ -1480,7 +1495,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>87</v>
       </c>
@@ -1500,7 +1515,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>87</v>
       </c>
@@ -1520,7 +1535,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>87</v>
       </c>
@@ -1540,7 +1555,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>87</v>
       </c>

</xml_diff>

<commit_message>
31052026 h1050: date fix in program.xlsx
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nontr\Documents\pisa-conf\ftdm26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3233526A-8CAD-4AB2-B08F-F9004E855DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE17DBA-0EF0-487E-9DE0-708C1C249714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="83">
   <si>
     <t>Key</t>
   </si>
@@ -260,6 +260,18 @@
   </si>
   <si>
     <t>Forum on Tracking Detector Mechanics</t>
+  </si>
+  <si>
+    <t>2026-06-01</t>
+  </si>
+  <si>
+    <t>2026-06-05</t>
+  </si>
+  <si>
+    <t>2026-06-01 07:00:00</t>
+  </si>
+  <si>
+    <t>2026-06-05 20:00:00</t>
   </si>
 </sst>
 </file>
@@ -318,13 +330,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -664,16 +675,16 @@
       <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2">
-        <v>46174</v>
+      <c r="B4" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2">
-        <v>46178</v>
+      <c r="B5" s="2" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -712,11 +723,11 @@
       <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="3">
-        <v>46174.291666666664</v>
-      </c>
-      <c r="D2" s="3">
-        <v>46178.833333333336</v>
+      <c r="C2" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
31052026 h1100: poster session start date adjusted
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nontr\Documents\pisa-conf\ftdm26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE17DBA-0EF0-487E-9DE0-708C1C249714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC0144B6-2BA2-4969-8DF2-A5BD55CABB88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -259,19 +259,19 @@
     <t>Universita' e INFN, Perugia (IT)</t>
   </si>
   <si>
-    <t>Forum on Tracking Detector Mechanics</t>
-  </si>
-  <si>
     <t>2026-06-01</t>
   </si>
   <si>
     <t>2026-06-05</t>
   </si>
   <si>
-    <t>2026-06-01 07:00:00</t>
-  </si>
-  <si>
     <t>2026-06-05 20:00:00</t>
+  </si>
+  <si>
+    <t>Forum on Tracking Detector Mechanics 2026</t>
+  </si>
+  <si>
+    <t>2026-05-31 07:00:00</t>
   </si>
 </sst>
 </file>
@@ -660,7 +660,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
@@ -676,7 +676,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
@@ -684,7 +684,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -724,10 +724,10 @@
         <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
31052026 h1200: adjust institution name to fit
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nontr\Documents\pisa-conf\ftdm26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC0144B6-2BA2-4969-8DF2-A5BD55CABB88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1929F88-0419-4E64-A757-2064D5F8F084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Conference" sheetId="1" r:id="rId1"/>
@@ -145,18 +145,12 @@
     <t>Grygiel</t>
   </si>
   <si>
-    <t>EPFL - Ecole Polytechnique Federale Lausanne (CH)</t>
-  </si>
-  <si>
     <t>CERN</t>
   </si>
   <si>
     <t>Rudjer Boskovic Institute (HR)</t>
   </si>
   <si>
-    <t>Deutsches Elektronen-Synchrotron  (DE)</t>
-  </si>
-  <si>
     <t>pi5pm1</t>
   </si>
   <si>
@@ -247,9 +241,6 @@
     <t>Wladyslaw Szczyrbak</t>
   </si>
   <si>
-    <t>Tadeusz Kosciuszko Cracow University of Technology (PL)</t>
-  </si>
-  <si>
     <t>Pier Filippo</t>
   </si>
   <si>
@@ -272,6 +263,15 @@
   </si>
   <si>
     <t>2026-05-31 07:00:00</t>
+  </si>
+  <si>
+    <t>Cracow University of Technology (PL)</t>
+  </si>
+  <si>
+    <t>DESY Hamburg (DE)</t>
+  </si>
+  <si>
+    <t>EPFL, Lausanne (CH)</t>
   </si>
 </sst>
 </file>
@@ -660,7 +660,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
@@ -676,7 +676,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
@@ -684,7 +684,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -724,10 +724,10 @@
         <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -753,7 +753,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -761,7 +761,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -769,7 +769,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -777,7 +777,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B5">
         <v>4</v>
@@ -785,7 +785,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -793,7 +793,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B7">
         <v>6</v>
@@ -801,7 +801,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B8">
         <v>7</v>
@@ -809,7 +809,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B9">
         <v>8</v>
@@ -817,7 +817,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B10">
         <v>9</v>
@@ -825,7 +825,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -833,7 +833,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -841,7 +841,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B13">
         <v>12</v>
@@ -849,7 +849,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B14">
         <v>13</v>
@@ -857,7 +857,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B15">
         <v>14</v>
@@ -865,7 +865,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B16">
         <v>15</v>
@@ -873,7 +873,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B17">
         <v>16</v>
@@ -881,7 +881,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B18">
         <v>17</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B19">
         <v>18</v>
@@ -897,7 +897,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B20">
         <v>19</v>
@@ -905,7 +905,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B21">
         <v>20</v>
@@ -913,7 +913,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B22">
         <v>21</v>
@@ -921,7 +921,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B23">
         <v>22</v>
@@ -929,7 +929,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B24">
         <v>23</v>
@@ -937,7 +937,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B25">
         <v>24</v>
@@ -945,7 +945,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B26">
         <v>25</v>
@@ -953,7 +953,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B27">
         <v>26</v>
@@ -961,7 +961,7 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B28">
         <v>27</v>
@@ -969,7 +969,7 @@
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B29">
         <v>28</v>
@@ -1028,7 +1028,7 @@
         <v>33</v>
       </c>
       <c r="F2" t="s">
-        <v>40</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
@@ -1048,7 +1048,7 @@
         <v>33</v>
       </c>
       <c r="F3" t="s">
-        <v>40</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
@@ -1068,7 +1068,7 @@
         <v>33</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
@@ -1088,7 +1088,7 @@
         <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
@@ -1108,7 +1108,7 @@
         <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
@@ -1128,7 +1128,7 @@
         <v>34</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
@@ -1148,7 +1148,7 @@
         <v>34</v>
       </c>
       <c r="F8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
@@ -1168,7 +1168,7 @@
         <v>34</v>
       </c>
       <c r="F9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
@@ -1188,7 +1188,7 @@
         <v>35</v>
       </c>
       <c r="F10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
@@ -1208,7 +1208,7 @@
         <v>35</v>
       </c>
       <c r="F11" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
@@ -1228,7 +1228,7 @@
         <v>35</v>
       </c>
       <c r="F12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
@@ -1248,7 +1248,7 @@
         <v>35</v>
       </c>
       <c r="F13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
@@ -1268,7 +1268,7 @@
         <v>36</v>
       </c>
       <c r="F14" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
@@ -1288,7 +1288,7 @@
         <v>36</v>
       </c>
       <c r="F15" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
@@ -1302,13 +1302,13 @@
         <v>22</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E16" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.45">
@@ -1322,13 +1322,13 @@
         <v>22</v>
       </c>
       <c r="D17" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.45">
@@ -1348,7 +1348,7 @@
         <v>37</v>
       </c>
       <c r="F18" t="s">
-        <v>43</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.45">
@@ -1368,7 +1368,7 @@
         <v>37</v>
       </c>
       <c r="F19" t="s">
-        <v>43</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.45">
@@ -1388,7 +1388,7 @@
         <v>37</v>
       </c>
       <c r="F20" t="s">
-        <v>43</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.45">
@@ -1408,7 +1408,7 @@
         <v>37</v>
       </c>
       <c r="F21" t="s">
-        <v>43</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.45">
@@ -1428,7 +1428,7 @@
         <v>38</v>
       </c>
       <c r="F22" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.45">
@@ -1448,7 +1448,7 @@
         <v>38</v>
       </c>
       <c r="F23" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.45">
@@ -1462,13 +1462,13 @@
         <v>24</v>
       </c>
       <c r="D24" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E24" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F24" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.45">
@@ -1482,13 +1482,13 @@
         <v>24</v>
       </c>
       <c r="D25" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E25" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F25" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.45">
@@ -1508,7 +1508,7 @@
         <v>39</v>
       </c>
       <c r="F26" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.45">
@@ -1528,7 +1528,7 @@
         <v>39</v>
       </c>
       <c r="F27" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.45">
@@ -1548,7 +1548,7 @@
         <v>39</v>
       </c>
       <c r="F28" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.45">
@@ -1568,7 +1568,7 @@
         <v>39</v>
       </c>
       <c r="F29" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
31052026 h1210: minor adjustments
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nontr\Documents\pisa-conf\ftdm26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1929F88-0419-4E64-A757-2064D5F8F084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58672FD-FACF-48C9-A124-8ED12A417621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -265,13 +265,13 @@
     <t>2026-05-31 07:00:00</t>
   </si>
   <si>
-    <t>Cracow University of Technology (PL)</t>
-  </si>
-  <si>
-    <t>DESY Hamburg (DE)</t>
-  </si>
-  <si>
     <t>EPFL, Lausanne (CH)</t>
+  </si>
+  <si>
+    <t>DESY, Hamburg (DE)</t>
+  </si>
+  <si>
+    <t>Politechnika Krakowska, Cracow (PL)</t>
   </si>
 </sst>
 </file>
@@ -1028,7 +1028,7 @@
         <v>33</v>
       </c>
       <c r="F2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
@@ -1048,7 +1048,7 @@
         <v>33</v>
       </c>
       <c r="F3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
@@ -1068,7 +1068,7 @@
         <v>33</v>
       </c>
       <c r="F4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
@@ -1088,7 +1088,7 @@
         <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
@@ -1468,7 +1468,7 @@
         <v>71</v>
       </c>
       <c r="F24" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.45">
@@ -1488,7 +1488,7 @@
         <v>71</v>
       </c>
       <c r="F25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
31052026 h1215: minor adjustments
</commit_message>
<xml_diff>
--- a/program.xlsx
+++ b/program.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nontr\Documents\pisa-conf\ftdm26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58672FD-FACF-48C9-A124-8ED12A417621}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CA3212F-4024-42D5-B2AE-0278C5F44A0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -271,7 +271,7 @@
     <t>DESY, Hamburg (DE)</t>
   </si>
   <si>
-    <t>Politechnika Krakowska, Cracow (PL)</t>
+    <t>PK/CUT, Cracow (PL)</t>
   </si>
 </sst>
 </file>

</xml_diff>